<commit_message>
Configure backend with Aiven MySQL
</commit_message>
<xml_diff>
--- a/commune.xlsx
+++ b/commune.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\ProjetJSAvancé\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16187DBC-EFCB-46F6-81ED-4DE73F56F131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F49F5E-859F-49B9-B6FB-A73324255207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="78">
   <si>
     <t>code_commune</t>
   </si>
@@ -33,21 +33,12 @@
     <t>nom_commune</t>
   </si>
   <si>
-    <t>nom_cisco</t>
-  </si>
-  <si>
     <t>CU FIANARANTSOA</t>
   </si>
   <si>
-    <t>FIANARANTSOA I</t>
-  </si>
-  <si>
     <t>ALAKAMISY AMBOHIMAHA</t>
   </si>
   <si>
-    <t>LALANGINA</t>
-  </si>
-  <si>
     <t>ALATSINAINY IALAMARINA</t>
   </si>
   <si>
@@ -195,9 +186,6 @@
     <t>TSITONDROINA</t>
   </si>
   <si>
-    <t>ISANDRA</t>
-  </si>
-  <si>
     <t>AMBALAMIDERA II</t>
   </si>
   <si>
@@ -228,9 +216,6 @@
     <t>MAHAZOARIVO</t>
   </si>
   <si>
-    <t>VOHIBATO</t>
-  </si>
-  <si>
     <t>ALAKAMISY ITENINA</t>
   </si>
   <si>
@@ -271,6 +256,9 @@
   </si>
   <si>
     <t>VOHITRAFENO</t>
+  </si>
+  <si>
+    <t>code_cisco</t>
   </si>
 </sst>
 </file>
@@ -616,7 +604,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -624,10 +612,10 @@
         <v>30101</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C2" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -635,10 +623,10 @@
         <v>30101</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C3" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -646,10 +634,10 @@
         <v>30101</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C4" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -657,10 +645,10 @@
         <v>30101</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C5" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -668,10 +656,10 @@
         <v>30101</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C6" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -679,10 +667,10 @@
         <v>30101</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C7" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -690,10 +678,10 @@
         <v>30101</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C8" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -701,10 +689,10 @@
         <v>30101</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C9" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -712,10 +700,10 @@
         <v>30101</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C10" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -723,10 +711,10 @@
         <v>30101</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C11" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -734,10 +722,10 @@
         <v>30101</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C12" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -745,10 +733,10 @@
         <v>30101</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C13" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -756,10 +744,10 @@
         <v>30101</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C14" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -767,10 +755,10 @@
         <v>30101</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C15" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -778,10 +766,10 @@
         <v>30101</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C16" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -789,10 +777,10 @@
         <v>30101</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C17" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -800,10 +788,10 @@
         <v>30101</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C18" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -811,10 +799,10 @@
         <v>30101</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C19" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -822,10 +810,10 @@
         <v>30101</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C20" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -833,10 +821,10 @@
         <v>30101</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C21" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -844,10 +832,10 @@
         <v>30101</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C22" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -855,10 +843,10 @@
         <v>30101</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C23" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -866,10 +854,10 @@
         <v>30101</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C24" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -877,10 +865,10 @@
         <v>30101</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C25" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -888,10 +876,10 @@
         <v>30101</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C26" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -899,10 +887,10 @@
         <v>30101</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C27" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -910,10 +898,10 @@
         <v>30101</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C28" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -921,10 +909,10 @@
         <v>30101</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C29" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -932,10 +920,10 @@
         <v>30101</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C30" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -943,10 +931,10 @@
         <v>30101</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C31" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -954,10 +942,10 @@
         <v>30101</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C32" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -965,10 +953,10 @@
         <v>30101</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C33" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -976,10 +964,10 @@
         <v>30101</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C34" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -987,10 +975,10 @@
         <v>30101</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C35" s="2">
+        <v>301</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -998,10 +986,10 @@
         <v>30201</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C36" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1009,10 +997,10 @@
         <v>30201</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C37" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1020,10 +1008,10 @@
         <v>30201</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C38" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1031,10 +1019,10 @@
         <v>30201</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C39" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1042,10 +1030,10 @@
         <v>30201</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C40" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1053,10 +1041,10 @@
         <v>30201</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C41" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1064,10 +1052,10 @@
         <v>30201</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C42" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1075,10 +1063,10 @@
         <v>30201</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C43" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1086,10 +1074,10 @@
         <v>30201</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C44" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1097,10 +1085,10 @@
         <v>30201</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C45" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1108,10 +1096,10 @@
         <v>30201</v>
       </c>
       <c r="B46" t="s">
-        <v>5</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C46" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1119,10 +1107,10 @@
         <v>30201</v>
       </c>
       <c r="B47" t="s">
-        <v>5</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="C47" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1130,10 +1118,10 @@
         <v>30203</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C48" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1141,10 +1129,10 @@
         <v>30203</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C49" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1152,10 +1140,10 @@
         <v>30203</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C50" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1163,10 +1151,10 @@
         <v>30203</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C51" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1174,10 +1162,10 @@
         <v>30203</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C52" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1185,10 +1173,10 @@
         <v>30203</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C53" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1196,10 +1184,10 @@
         <v>30203</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C54" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1207,10 +1195,10 @@
         <v>30203</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C55" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1218,10 +1206,10 @@
         <v>30203</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C56" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1229,10 +1217,10 @@
         <v>30203</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="C57" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1240,10 +1228,10 @@
         <v>30204</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C58" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1251,10 +1239,10 @@
         <v>30204</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C59" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1262,10 +1250,10 @@
         <v>30204</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C60" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1273,10 +1261,10 @@
         <v>30204</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C61" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1284,10 +1272,10 @@
         <v>30204</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C62" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1295,10 +1283,10 @@
         <v>30204</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C63" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1306,10 +1294,10 @@
         <v>30204</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="C64" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1317,10 +1305,10 @@
         <v>30205</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C65" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C65" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1328,10 +1316,10 @@
         <v>30205</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C66" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C66" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1339,10 +1327,10 @@
         <v>30205</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C67" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C67" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1350,10 +1338,10 @@
         <v>30205</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C68" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C68" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1361,10 +1349,10 @@
         <v>30205</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C69" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C69" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1372,10 +1360,10 @@
         <v>30205</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C70" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C70" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1383,10 +1371,10 @@
         <v>30205</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C71" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C71" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1394,10 +1382,10 @@
         <v>30205</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C72" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C72" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1405,10 +1393,10 @@
         <v>30209</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C73" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1416,10 +1404,10 @@
         <v>30209</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C74" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1427,10 +1415,10 @@
         <v>30209</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C75" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1438,10 +1426,10 @@
         <v>30209</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C76" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1449,10 +1437,10 @@
         <v>30209</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C77" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1460,10 +1448,10 @@
         <v>30209</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C78" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1471,10 +1459,10 @@
         <v>30212</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C79" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1482,10 +1470,10 @@
         <v>30212</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C80" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1493,10 +1481,10 @@
         <v>30212</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C81" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1504,10 +1492,10 @@
         <v>30212</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C82" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="83" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1515,10 +1503,10 @@
         <v>30212</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C83" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="84" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1526,10 +1514,10 @@
         <v>30212</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C84" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1537,10 +1525,10 @@
         <v>30212</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C85" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="86" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1548,10 +1536,10 @@
         <v>30212</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C86" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1559,10 +1547,10 @@
         <v>30212</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C87" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1570,10 +1558,10 @@
         <v>30212</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C88" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="89" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1581,10 +1569,10 @@
         <v>30212</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C89" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="90" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1592,10 +1580,10 @@
         <v>30212</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C90" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1603,10 +1591,10 @@
         <v>30212</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C91" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="92" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1614,10 +1602,10 @@
         <v>30212</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C92" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="93" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1625,10 +1613,10 @@
         <v>30212</v>
       </c>
       <c r="B93" t="s">
-        <v>11</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C93" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1636,10 +1624,10 @@
         <v>30212</v>
       </c>
       <c r="B94" t="s">
-        <v>11</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C94" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1647,10 +1635,10 @@
         <v>30215</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="C95" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="96" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1658,10 +1646,10 @@
         <v>30215</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="C96" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="97" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1669,10 +1657,10 @@
         <v>30215</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="C97" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="98" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1680,10 +1668,10 @@
         <v>30215</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="C98" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1691,10 +1679,10 @@
         <v>30238</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C99" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="100" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1702,10 +1690,10 @@
         <v>30238</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C100" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1713,10 +1701,10 @@
         <v>30238</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C101" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="102" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1724,10 +1712,10 @@
         <v>30238</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C102" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="103" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1735,10 +1723,10 @@
         <v>30238</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C103" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="104" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1746,10 +1734,10 @@
         <v>30242</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="C104" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="105" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1757,10 +1745,10 @@
         <v>30243</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
+      </c>
+      <c r="C105" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1768,10 +1756,10 @@
         <v>30244</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
+      </c>
+      <c r="C106" s="2">
+        <v>302</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1779,10 +1767,10 @@
         <v>30245</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
+      </c>
+      <c r="C107" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="108" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1790,10 +1778,10 @@
         <v>30248</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
+      </c>
+      <c r="C108" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="109" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1801,10 +1789,10 @@
         <v>30301</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
+      </c>
+      <c r="C109" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1812,10 +1800,10 @@
         <v>30303</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="C110" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1823,10 +1811,10 @@
         <v>30304</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="C111" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1834,10 +1822,10 @@
         <v>30305</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C112" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="C112" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1845,10 +1833,10 @@
         <v>30306</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="C113" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="114" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1856,10 +1844,10 @@
         <v>30307</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="C114" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1867,10 +1855,10 @@
         <v>30308</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="C115" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1878,10 +1866,10 @@
         <v>30309</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
+      </c>
+      <c r="C116" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1889,10 +1877,10 @@
         <v>30310</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C117" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
+      </c>
+      <c r="C117" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="118" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1900,10 +1888,10 @@
         <v>30311</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>19</v>
+        <v>25</v>
+      </c>
+      <c r="C118" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="119" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1911,10 +1899,10 @@
         <v>30319</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="C119" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1922,10 +1910,10 @@
         <v>30312</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
+      </c>
+      <c r="C120" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="121" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1933,10 +1921,10 @@
         <v>30313</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C121" s="2" t="s">
-        <v>19</v>
+        <v>28</v>
+      </c>
+      <c r="C121" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1944,10 +1932,10 @@
         <v>30314</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>19</v>
+        <v>29</v>
+      </c>
+      <c r="C122" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1955,10 +1943,10 @@
         <v>30315</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>19</v>
+        <v>30</v>
+      </c>
+      <c r="C123" s="2">
+        <v>303</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1966,10 +1954,10 @@
         <v>30503</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
+      </c>
+      <c r="C124" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1977,10 +1965,10 @@
         <v>30504</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="C125" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1988,10 +1976,10 @@
         <v>30505</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
+      </c>
+      <c r="C126" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1999,10 +1987,10 @@
         <v>30506</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C127" s="2" t="s">
         <v>34</v>
+      </c>
+      <c r="C127" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2010,10 +1998,10 @@
         <v>30507</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="C128" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2021,10 +2009,10 @@
         <v>30508</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
+      </c>
+      <c r="C129" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="130" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2032,10 +2020,10 @@
         <v>30509</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="C130" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="131" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2043,10 +2031,10 @@
         <v>30510</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C131" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
+      </c>
+      <c r="C131" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="132" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2054,10 +2042,10 @@
         <v>30511</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C132" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
+      </c>
+      <c r="C132" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="133" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2065,10 +2053,10 @@
         <v>30512</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C133" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
+      </c>
+      <c r="C133" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="134" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2076,10 +2064,10 @@
         <v>30513</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>34</v>
+        <v>41</v>
+      </c>
+      <c r="C134" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="135" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2087,10 +2075,10 @@
         <v>30514</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="C135" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="136" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2098,10 +2086,10 @@
         <v>30515</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C136" s="2" t="s">
-        <v>34</v>
+        <v>43</v>
+      </c>
+      <c r="C136" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="137" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2109,10 +2097,10 @@
         <v>30517</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="C137" s="2">
+        <v>304</v>
       </c>
     </row>
     <row r="138" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2120,10 +2108,10 @@
         <v>31401</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="C138" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="139" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2131,10 +2119,10 @@
         <v>31402</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
+      </c>
+      <c r="C139" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="140" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2142,10 +2130,10 @@
         <v>31403</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C140" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
+      </c>
+      <c r="C140" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="141" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2153,10 +2141,10 @@
         <v>31404</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C141" s="2" t="s">
         <v>48</v>
+      </c>
+      <c r="C141" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="142" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2164,10 +2152,10 @@
         <v>31405</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="C142" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="143" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2175,10 +2163,10 @@
         <v>31406</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="C143" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="144" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2186,10 +2174,10 @@
         <v>31407</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
+      </c>
+      <c r="C144" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="145" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2197,10 +2185,10 @@
         <v>31408</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
+      </c>
+      <c r="C145" s="2">
+        <v>314</v>
       </c>
     </row>
     <row r="146" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2208,10 +2196,10 @@
         <v>32501</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
+      </c>
+      <c r="C146" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="147" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2219,10 +2207,10 @@
         <v>32502</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
+      </c>
+      <c r="C147" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="148" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2230,10 +2218,10 @@
         <v>32503</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C148" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="C148" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="149" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2241,10 +2229,10 @@
         <v>32504</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C149" s="2" t="s">
         <v>56</v>
+      </c>
+      <c r="C149" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="150" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2252,10 +2240,10 @@
         <v>32505</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C150" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="C150" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="151" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2263,10 +2251,10 @@
         <v>32513</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C151" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
+      </c>
+      <c r="C151" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="152" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2274,10 +2262,10 @@
         <v>32506</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
+      </c>
+      <c r="C152" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="153" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2285,10 +2273,10 @@
         <v>32508</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
+      </c>
+      <c r="C153" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="154" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2296,10 +2284,10 @@
         <v>32512</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
+      </c>
+      <c r="C154" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="155" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2307,10 +2295,10 @@
         <v>32509</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>56</v>
+        <v>62</v>
+      </c>
+      <c r="C155" s="2">
+        <v>325</v>
       </c>
     </row>
     <row r="156" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2318,10 +2306,10 @@
         <v>32601</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C156" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
+      </c>
+      <c r="C156" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="157" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2329,10 +2317,10 @@
         <v>32602</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C157" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
+      </c>
+      <c r="C157" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="158" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2340,10 +2328,10 @@
         <v>32603</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
+      </c>
+      <c r="C158" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="159" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2351,10 +2339,10 @@
         <v>32604</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C159" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
+      </c>
+      <c r="C159" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="160" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2362,10 +2350,10 @@
         <v>32605</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C160" s="2" t="s">
         <v>67</v>
+      </c>
+      <c r="C160" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="161" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2373,10 +2361,10 @@
         <v>32606</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C161" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
+      </c>
+      <c r="C161" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="162" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2384,10 +2372,10 @@
         <v>32615</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C162" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+      <c r="C162" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="163" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2395,10 +2383,10 @@
         <v>32608</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C163" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
+      </c>
+      <c r="C163" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="164" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2406,10 +2394,10 @@
         <v>32609</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C164" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
+      </c>
+      <c r="C164" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="165" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2417,10 +2405,10 @@
         <v>32610</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C165" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
+      </c>
+      <c r="C165" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="166" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2428,10 +2416,10 @@
         <v>32611</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C166" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
+      </c>
+      <c r="C166" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="167" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2439,10 +2427,10 @@
         <v>32613</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C167" s="2" t="s">
-        <v>67</v>
+        <v>74</v>
+      </c>
+      <c r="C167" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="168" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2450,10 +2438,10 @@
         <v>32616</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C168" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
+      </c>
+      <c r="C168" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="169" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -2461,16 +2449,14 @@
         <v>32614</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C169" s="2" t="s">
-        <v>67</v>
+        <v>76</v>
+      </c>
+      <c r="C169" s="2">
+        <v>326</v>
       </c>
     </row>
     <row r="170" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="C170" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="C170" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>